<commit_message>
New calcium peak finder
Minimum 3 peaks, picks 1 in middle
</commit_message>
<xml_diff>
--- a/For Drug Challenge/Simulation_Results_Log.xlsx
+++ b/For Drug Challenge/Simulation_Results_Log.xlsx
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U11"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.21875" customWidth="true"/>
@@ -1198,6 +1198,136 @@
         <v>2767.5256230875475</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="0">
+        <v>4</v>
+      </c>
+      <c r="B12" s="0">
+        <v>1</v>
+      </c>
+      <c r="C12" s="0">
+        <v>10</v>
+      </c>
+      <c r="D12" s="0">
+        <v>52.813785983823543</v>
+      </c>
+      <c r="E12" s="0">
+        <v>569.71450534793803</v>
+      </c>
+      <c r="F12" s="0">
+        <v>226.70093110920425</v>
+      </c>
+      <c r="G12" s="0">
+        <v>66.0259501317569</v>
+      </c>
+      <c r="H12" s="0">
+        <v>26.380314939850237</v>
+      </c>
+      <c r="I12" s="0">
+        <v>7.5937349283928661</v>
+      </c>
+      <c r="J12" s="0">
+        <v>540.35338323200961</v>
+      </c>
+      <c r="K12" s="0">
+        <v>540.36980386814605</v>
+      </c>
+      <c r="L12" s="0">
+        <v>0.83294297381631766</v>
+      </c>
+      <c r="M12" s="0">
+        <v>0.16705702618368234</v>
+      </c>
+      <c r="N12" s="0">
+        <v>0.89005610660786549</v>
+      </c>
+      <c r="O12" s="0">
+        <v>-75.726647237186711</v>
+      </c>
+      <c r="P12" s="0">
+        <v>114.68444047216002</v>
+      </c>
+      <c r="Q12" s="0">
+        <v>38.957793234973302</v>
+      </c>
+      <c r="R12" s="0">
+        <v>127.93451211941007</v>
+      </c>
+      <c r="S12" s="0">
+        <v>2467.993240405478</v>
+      </c>
+      <c r="T12" s="0">
+        <v>2657.6439481351917</v>
+      </c>
+      <c r="U12" s="0">
+        <v>2767.5256230875475</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0">
+        <v>4</v>
+      </c>
+      <c r="B13" s="0">
+        <v>1</v>
+      </c>
+      <c r="C13" s="0">
+        <v>10</v>
+      </c>
+      <c r="D13" s="0">
+        <v>52.792401451961538</v>
+      </c>
+      <c r="E13" s="0">
+        <v>569.26304975057553</v>
+      </c>
+      <c r="F13" s="0">
+        <v>227.06954161488375</v>
+      </c>
+      <c r="G13" s="0">
+        <v>62.797752439863572</v>
+      </c>
+      <c r="H13" s="0">
+        <v>29.531744147006233</v>
+      </c>
+      <c r="I13" s="0">
+        <v>7.6705034131301826</v>
+      </c>
+      <c r="J13" s="0">
+        <v>434.95634414083776</v>
+      </c>
+      <c r="K13" s="0">
+        <v>434.96314968078821</v>
+      </c>
+      <c r="L13" s="0">
+        <v>0.57331737923927473</v>
+      </c>
+      <c r="M13" s="0">
+        <v>0.42668262076072527</v>
+      </c>
+      <c r="N13" s="0">
+        <v>0.90655680566951558</v>
+      </c>
+      <c r="O13" s="0">
+        <v>-75.726647237186711</v>
+      </c>
+      <c r="P13" s="0">
+        <v>114.68444047216002</v>
+      </c>
+      <c r="Q13" s="0">
+        <v>38.957793234973302</v>
+      </c>
+      <c r="R13" s="0">
+        <v>127.93451211941007</v>
+      </c>
+      <c r="S13" s="0">
+        <v>2467.993240405478</v>
+      </c>
+      <c r="T13" s="0">
+        <v>2657.6439481351917</v>
+      </c>
+      <c r="U13" s="0">
+        <v>2767.5256230875475</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed APD Grouped Trace bug
</commit_message>
<xml_diff>
--- a/For Drug Challenge/Simulation_Results_Log.xlsx
+++ b/For Drug Challenge/Simulation_Results_Log.xlsx
@@ -457,7 +457,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U13"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="6.21875" customWidth="true"/>
@@ -466,8 +466,8 @@
     <col min="4" max="4" width="14.33203125" customWidth="true"/>
     <col min="5" max="5" width="11.5546875" customWidth="true"/>
     <col min="11" max="11" width="11.77734375" customWidth="true"/>
-    <col min="12" max="12" width="13.5546875" customWidth="true"/>
-    <col min="13" max="13" width="12.5546875" customWidth="true"/>
+    <col min="12" max="12" width="15.5546875" customWidth="true"/>
+    <col min="13" max="13" width="15.5546875" customWidth="true"/>
     <col min="14" max="14" width="18.5546875" customWidth="true"/>
     <col min="15" max="15" width="12.21875" customWidth="true"/>
     <col min="16" max="16" width="11.5546875" customWidth="true"/>
@@ -1328,6 +1328,396 @@
         <v>2767.5256230875475</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" s="0">
+        <v>4</v>
+      </c>
+      <c r="B14" s="0">
+        <v>1</v>
+      </c>
+      <c r="C14" s="0">
+        <v>10</v>
+      </c>
+      <c r="D14" s="0">
+        <v>52.7957054202259</v>
+      </c>
+      <c r="E14" s="0">
+        <v>569.71450534793803</v>
+      </c>
+      <c r="F14" s="0">
+        <v>226.70093110920425</v>
+      </c>
+      <c r="G14" s="0">
+        <v>62.759924633748618</v>
+      </c>
+      <c r="H14" s="0">
+        <v>29.574704696271819</v>
+      </c>
+      <c r="I14" s="0">
+        <v>7.6653706699795636</v>
+      </c>
+      <c r="J14" s="0">
+        <v>435.04092841277804</v>
+      </c>
+      <c r="K14" s="0">
+        <v>435.19172903845305</v>
+      </c>
+      <c r="L14" s="0">
+        <v>0.56841519913478067</v>
+      </c>
+      <c r="M14" s="0">
+        <v>0.43158480086521933</v>
+      </c>
+      <c r="N14" s="0">
+        <v>0.90696978246767013</v>
+      </c>
+      <c r="O14" s="0">
+        <v>-75.726647237186711</v>
+      </c>
+      <c r="P14" s="0">
+        <v>114.658369300025</v>
+      </c>
+      <c r="Q14" s="0">
+        <v>38.93172206283829</v>
+      </c>
+      <c r="R14" s="0">
+        <v>127.93451211941007</v>
+      </c>
+      <c r="S14" s="0">
+        <v>465.99176041045484</v>
+      </c>
+      <c r="T14" s="0">
+        <v>655.54505633357621</v>
+      </c>
+      <c r="U14" s="0">
+        <v>765.27259589526784</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0">
+        <v>4</v>
+      </c>
+      <c r="B15" s="0">
+        <v>1</v>
+      </c>
+      <c r="C15" s="0">
+        <v>10</v>
+      </c>
+      <c r="D15" s="0">
+        <v>52.7957054202259</v>
+      </c>
+      <c r="E15" s="0">
+        <v>569.71450534793803</v>
+      </c>
+      <c r="F15" s="0">
+        <v>226.70093110920425</v>
+      </c>
+      <c r="G15" s="0">
+        <v>62.759924633748618</v>
+      </c>
+      <c r="H15" s="0">
+        <v>29.574704696271819</v>
+      </c>
+      <c r="I15" s="0">
+        <v>7.6653706699795636</v>
+      </c>
+      <c r="J15" s="0">
+        <v>435.04092841277804</v>
+      </c>
+      <c r="K15" s="0">
+        <v>435.19172903845305</v>
+      </c>
+      <c r="L15" s="0">
+        <v>0.56841519913478067</v>
+      </c>
+      <c r="M15" s="0">
+        <v>0.43158480086521933</v>
+      </c>
+      <c r="N15" s="0">
+        <v>0.90696978246767013</v>
+      </c>
+      <c r="O15" s="0">
+        <v>-75.726647237186711</v>
+      </c>
+      <c r="P15" s="0">
+        <v>114.74741048291276</v>
+      </c>
+      <c r="Q15" s="0">
+        <v>39.020763245726037</v>
+      </c>
+      <c r="R15" s="0">
+        <v>127.93451211941007</v>
+      </c>
+      <c r="S15" s="0">
+        <v>4467.6248676215509</v>
+      </c>
+      <c r="T15" s="0">
+        <v>4657.9562975431854</v>
+      </c>
+      <c r="U15" s="0">
+        <v>4768.2166551196733</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0">
+        <v>4</v>
+      </c>
+      <c r="B16" s="0">
+        <v>1</v>
+      </c>
+      <c r="C16" s="0">
+        <v>10</v>
+      </c>
+      <c r="D16" s="0">
+        <v>52.7957054202259</v>
+      </c>
+      <c r="E16" s="0">
+        <v>569.71450534793803</v>
+      </c>
+      <c r="F16" s="0">
+        <v>226.70093110920425</v>
+      </c>
+      <c r="G16" s="0">
+        <v>62.759924633748618</v>
+      </c>
+      <c r="H16" s="0">
+        <v>29.574704696271819</v>
+      </c>
+      <c r="I16" s="0">
+        <v>7.6653706699795636</v>
+      </c>
+      <c r="J16" s="0">
+        <v>435.04092841277804</v>
+      </c>
+      <c r="K16" s="0">
+        <v>435.19172903845305</v>
+      </c>
+      <c r="L16" s="0">
+        <v>0.56841519913478067</v>
+      </c>
+      <c r="M16" s="0">
+        <v>0.43158480086521933</v>
+      </c>
+      <c r="N16" s="0">
+        <v>0.90696978246767013</v>
+      </c>
+      <c r="O16" s="0">
+        <v>-75.726647237186711</v>
+      </c>
+      <c r="P16" s="0">
+        <v>114.658369300025</v>
+      </c>
+      <c r="Q16" s="0">
+        <v>38.93172206283829</v>
+      </c>
+      <c r="R16" s="0">
+        <v>127.93451211941007</v>
+      </c>
+      <c r="S16" s="0">
+        <v>465.99176041045484</v>
+      </c>
+      <c r="T16" s="0">
+        <v>655.54505633357621</v>
+      </c>
+      <c r="U16" s="0">
+        <v>765.27259589526784</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0">
+        <v>4</v>
+      </c>
+      <c r="B17" s="0">
+        <v>1</v>
+      </c>
+      <c r="C17" s="0">
+        <v>10</v>
+      </c>
+      <c r="D17" s="0">
+        <v>52.7957054202259</v>
+      </c>
+      <c r="E17" s="0">
+        <v>569.71450534793803</v>
+      </c>
+      <c r="F17" s="0">
+        <v>226.70093110920425</v>
+      </c>
+      <c r="G17" s="0">
+        <v>62.759924633748618</v>
+      </c>
+      <c r="H17" s="0">
+        <v>29.574704696271819</v>
+      </c>
+      <c r="I17" s="0">
+        <v>7.6653706699795636</v>
+      </c>
+      <c r="J17" s="0">
+        <v>435.04092841277804</v>
+      </c>
+      <c r="K17" s="0">
+        <v>435.19172903845305</v>
+      </c>
+      <c r="L17" s="0">
+        <v>0.56841519913478067</v>
+      </c>
+      <c r="M17" s="0">
+        <v>0.43158480086521933</v>
+      </c>
+      <c r="N17" s="0">
+        <v>0.90696978246767013</v>
+      </c>
+      <c r="O17" s="0">
+        <v>-75.726647237186711</v>
+      </c>
+      <c r="P17" s="0">
+        <v>114.658369300025</v>
+      </c>
+      <c r="Q17" s="0">
+        <v>38.93172206283829</v>
+      </c>
+      <c r="R17" s="0">
+        <v>127.93451211941007</v>
+      </c>
+      <c r="S17" s="0">
+        <v>465.99176041045484</v>
+      </c>
+      <c r="T17" s="0">
+        <v>655.54505633357621</v>
+      </c>
+      <c r="U17" s="0">
+        <v>765.27259589526784</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>0</v>
+      </c>
+      <c r="B18" s="0">
+        <v>1</v>
+      </c>
+      <c r="C18" s="0">
+        <v>10</v>
+      </c>
+      <c r="D18" s="0">
+        <v>52.423897879396485</v>
+      </c>
+      <c r="E18" s="0">
+        <v>558.98163463424089</v>
+      </c>
+      <c r="F18" s="0">
+        <v>207.16911364893531</v>
+      </c>
+      <c r="G18" s="0">
+        <v>58.078230058856541</v>
+      </c>
+      <c r="H18" s="0">
+        <v>34.33191687218833</v>
+      </c>
+      <c r="I18" s="0">
+        <v>7.5898530689551365</v>
+      </c>
+      <c r="J18" s="0">
+        <v>294.0459577270916</v>
+      </c>
+      <c r="K18" s="0">
+        <v>294.04610323059131</v>
+      </c>
+      <c r="L18" s="0">
+        <v>0.00035894509320821832</v>
+      </c>
+      <c r="M18" s="0">
+        <v>0.99964105490679178</v>
+      </c>
+      <c r="N18" s="0">
+        <v>0.89752180991683594</v>
+      </c>
+      <c r="O18" s="0">
+        <v>-75.73917575411194</v>
+      </c>
+      <c r="P18" s="0">
+        <v>113.68590268996741</v>
+      </c>
+      <c r="Q18" s="0">
+        <v>37.946726935855466</v>
+      </c>
+      <c r="R18" s="0">
+        <v>134.69991731651683</v>
+      </c>
+      <c r="S18" s="0">
+        <v>336.37451649255672</v>
+      </c>
+      <c r="T18" s="0">
+        <v>401.33901247254289</v>
+      </c>
+      <c r="U18" s="0">
+        <v>443.10608322380904</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>0</v>
+      </c>
+      <c r="B19" s="0">
+        <v>1</v>
+      </c>
+      <c r="C19" s="0">
+        <v>5</v>
+      </c>
+      <c r="D19" s="0">
+        <v>52.393601198791146</v>
+      </c>
+      <c r="E19" s="0">
+        <v>560.23469367993721</v>
+      </c>
+      <c r="F19" s="0">
+        <v>206.82392782405259</v>
+      </c>
+      <c r="G19" s="0">
+        <v>58.090141682841512</v>
+      </c>
+      <c r="H19" s="0">
+        <v>34.323330318229772</v>
+      </c>
+      <c r="I19" s="0">
+        <v>7.586527998928724</v>
+      </c>
+      <c r="J19" s="0">
+        <v>294.03003381735476</v>
+      </c>
+      <c r="K19" s="0">
+        <v>300.04612901284111</v>
+      </c>
+      <c r="L19" s="0">
+        <v>0.99963856557421904</v>
+      </c>
+      <c r="M19" s="0">
+        <v>0.00036143442578095986</v>
+      </c>
+      <c r="N19" s="0">
+        <v>0.89731328156226975</v>
+      </c>
+      <c r="O19" s="0">
+        <v>-75.739175625440481</v>
+      </c>
+      <c r="P19" s="0">
+        <v>113.57898015447321</v>
+      </c>
+      <c r="Q19" s="0">
+        <v>37.839804529032726</v>
+      </c>
+      <c r="R19" s="0">
+        <v>133.59022835623125</v>
+      </c>
+      <c r="S19" s="0">
+        <v>337.9121898585372</v>
+      </c>
+      <c r="T19" s="0">
+        <v>403.08953885191977</v>
+      </c>
+      <c r="U19" s="0">
+        <v>445.15774089237721</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Overlay drug titers Nifedipine
</commit_message>
<xml_diff>
--- a/For Drug Challenge/Simulation_Results_Log.xlsx
+++ b/For Drug Challenge/Simulation_Results_Log.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -10,12 +10,12 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="4" documentId="11_324AE617CF19DF2F225B9B65E4012D160102563D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{61076E25-4958-4AFB-8AD8-B99E479DC21A}"/>
   <bookViews>
-    <workbookView xWindow="-31065" yWindow="9660" windowWidth="28020" windowHeight="14040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-31065" yWindow="9660" windowWidth="28020" windowHeight="14040"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="21" uniqueCount="21">
   <si>
     <t>Model</t>
   </si>
@@ -101,8 +101,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -116,7 +116,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -124,12 +124,14 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -152,7 +154,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -303,7 +305,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -327,9 +329,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -353,7 +355,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -388,7 +390,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -406,7 +408,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -431,7 +433,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -467,25 +469,34 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U30"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.21875" customWidth="1"/>
-    <col min="2" max="2" width="4.77734375" customWidth="1"/>
-    <col min="3" max="3" width="5.109375" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" customWidth="1"/>
-    <col min="5" max="10" width="11.5546875" customWidth="1"/>
-    <col min="11" max="11" width="11.77734375" customWidth="1"/>
-    <col min="12" max="13" width="15.5546875" customWidth="1"/>
-    <col min="14" max="14" width="18.5546875" customWidth="1"/>
-    <col min="15" max="15" width="12.21875" customWidth="1"/>
-    <col min="16" max="17" width="11.5546875" customWidth="1"/>
-    <col min="18" max="18" width="13.109375" customWidth="1"/>
-    <col min="19" max="21" width="11.5546875" customWidth="1"/>
+    <col min="1" max="1" width="6.21875" customWidth="true"/>
+    <col min="2" max="2" width="4.77734375" customWidth="true"/>
+    <col min="3" max="3" width="5.109375" customWidth="true"/>
+    <col min="4" max="4" width="14.33203125" customWidth="true"/>
+    <col min="5" max="5" width="11.5546875" customWidth="true"/>
+    <col min="11" max="11" width="11.77734375" customWidth="true"/>
+    <col min="12" max="12" width="15.5546875" customWidth="true"/>
+    <col min="14" max="14" width="18.5546875" customWidth="true"/>
+    <col min="15" max="15" width="12.21875" customWidth="true"/>
+    <col min="16" max="16" width="11.5546875" customWidth="true"/>
+    <col min="18" max="18" width="13.109375" customWidth="true"/>
+    <col min="19" max="19" width="11.5546875" customWidth="true"/>
+    <col min="6" max="6" width="11.5546875" customWidth="true"/>
+    <col min="7" max="7" width="11.5546875" customWidth="true"/>
+    <col min="8" max="8" width="11.5546875" customWidth="true"/>
+    <col min="9" max="9" width="11.5546875" customWidth="true"/>
+    <col min="10" max="10" width="11.5546875" customWidth="true"/>
+    <col min="13" max="13" width="15.5546875" customWidth="true"/>
+    <col min="17" max="17" width="11.5546875" customWidth="true"/>
+    <col min="20" max="20" width="11.5546875" customWidth="true"/>
+    <col min="21" max="21" width="11.5546875" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -550,7 +561,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>0</v>
       </c>
@@ -615,7 +626,7 @@
         <v>445.15774089237721</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>1</v>
       </c>
@@ -680,7 +691,7 @@
         <v>612.53106459655555</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>2</v>
       </c>
@@ -745,7 +756,7 @@
         <v>624.32699643900833</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>3</v>
       </c>
@@ -810,7 +821,7 @@
         <v>749.59288546012294</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>4</v>
       </c>
@@ -875,7 +886,7 @@
         <v>774.87230480672224</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>0</v>
       </c>
@@ -940,7 +951,7 @@
         <v>443.10608322380904</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1005,7 +1016,7 @@
         <v>612.01806178589959</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1070,7 +1081,7 @@
         <v>621.48202972051695</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>3</v>
       </c>
@@ -1135,7 +1146,7 @@
         <v>752.87191218775297</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>4</v>
       </c>
@@ -1200,7 +1211,7 @@
         <v>765.27259589526784</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>0</v>
       </c>
@@ -1265,7 +1276,7 @@
         <v>444.7117315806081</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>1</v>
       </c>
@@ -1330,7 +1341,7 @@
         <v>610.14847538790673</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1395,7 +1406,7 @@
         <v>620.08098036044885</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>3</v>
       </c>
@@ -1460,7 +1471,7 @@
         <v>743.75082824049787</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>4</v>
       </c>
@@ -1525,7 +1536,7 @@
         <v>763.740094575076</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>0</v>
       </c>
@@ -1590,7 +1601,7 @@
         <v>444.8873856820519</v>
       </c>
     </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>1</v>
       </c>
@@ -1655,7 +1666,7 @@
         <v>608.07351869433296</v>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>2</v>
       </c>
@@ -1720,7 +1731,7 @@
         <v>615.63409556269471</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>3</v>
       </c>
@@ -1785,7 +1796,7 @@
         <v>739.16884492881218</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>4</v>
       </c>
@@ -1848,6 +1859,591 @@
       </c>
       <c r="U21">
         <v>748.97339891578849</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0">
+        <v>4</v>
+      </c>
+      <c r="B22" s="0">
+        <v>2</v>
+      </c>
+      <c r="C22" s="0">
+        <v>100</v>
+      </c>
+      <c r="D22" s="0">
+        <v>42.913920157355903</v>
+      </c>
+      <c r="E22" s="0">
+        <v>244.14641275510769</v>
+      </c>
+      <c r="F22" s="0">
+        <v>156.84456525247788</v>
+      </c>
+      <c r="G22" s="0">
+        <v>55.503071008308602</v>
+      </c>
+      <c r="H22" s="0">
+        <v>35.918269146867452</v>
+      </c>
+      <c r="I22" s="0">
+        <v>8.5786598448239371</v>
+      </c>
+      <c r="J22" s="0">
+        <v>373.84958953975536</v>
+      </c>
+      <c r="K22" s="0">
+        <v>373.84966395888449</v>
+      </c>
+      <c r="L22" s="0">
+        <v>0.99186541242400694</v>
+      </c>
+      <c r="M22" s="0">
+        <v>0.0081345875759930575</v>
+      </c>
+      <c r="N22" s="0">
+        <v>0.93296967263549335</v>
+      </c>
+      <c r="O22" s="0">
+        <v>-75.728306505951252</v>
+      </c>
+      <c r="P22" s="0">
+        <v>102.22480007243072</v>
+      </c>
+      <c r="Q22" s="0">
+        <v>26.496493566479469</v>
+      </c>
+      <c r="R22" s="0">
+        <v>121.30415278154594</v>
+      </c>
+      <c r="S22" s="0">
+        <v>344.04932095109325</v>
+      </c>
+      <c r="T22" s="0">
+        <v>426.71008868054741</v>
+      </c>
+      <c r="U22" s="0">
+        <v>496.19891012479638</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0">
+        <v>4</v>
+      </c>
+      <c r="B23" s="0">
+        <v>2</v>
+      </c>
+      <c r="C23" s="0">
+        <v>200</v>
+      </c>
+      <c r="D23" s="0">
+        <v>40.42567114810447</v>
+      </c>
+      <c r="E23" s="0">
+        <v>189.35747153390992</v>
+      </c>
+      <c r="F23" s="0">
+        <v>161.36254074325825</v>
+      </c>
+      <c r="G23" s="0">
+        <v>51.860928961709973</v>
+      </c>
+      <c r="H23" s="0">
+        <v>39.135910252303098</v>
+      </c>
+      <c r="I23" s="0">
+        <v>9.0031607859869265</v>
+      </c>
+      <c r="J23" s="0">
+        <v>332.29777755356793</v>
+      </c>
+      <c r="K23" s="0">
+        <v>333.47099073068682</v>
+      </c>
+      <c r="L23" s="0">
+        <v>0.97268180479397892</v>
+      </c>
+      <c r="M23" s="0">
+        <v>0.027318195206021079</v>
+      </c>
+      <c r="N23" s="0">
+        <v>0.94184967215915594</v>
+      </c>
+      <c r="O23" s="0">
+        <v>-75.72842307261476</v>
+      </c>
+      <c r="P23" s="0">
+        <v>96.633452863376959</v>
+      </c>
+      <c r="Q23" s="0">
+        <v>20.905029790762196</v>
+      </c>
+      <c r="R23" s="0">
+        <v>124.052495517411</v>
+      </c>
+      <c r="S23" s="0">
+        <v>299.50625310685882</v>
+      </c>
+      <c r="T23" s="0">
+        <v>366.06246921662841</v>
+      </c>
+      <c r="U23" s="0">
+        <v>427.14435696349483</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0">
+        <v>4</v>
+      </c>
+      <c r="B24" s="0">
+        <v>1</v>
+      </c>
+      <c r="C24" s="0">
+        <v>15</v>
+      </c>
+      <c r="D24" s="0">
+        <v>51.825064679478217</v>
+      </c>
+      <c r="E24" s="0">
+        <v>576.27516495942029</v>
+      </c>
+      <c r="F24" s="0">
+        <v>205.81742929112625</v>
+      </c>
+      <c r="G24" s="0">
+        <v>56.998883955324231</v>
+      </c>
+      <c r="H24" s="0">
+        <v>34.971395564619314</v>
+      </c>
+      <c r="I24" s="0">
+        <v>8.0297204800564597</v>
+      </c>
+      <c r="J24" s="0">
+        <v>423.32078747809578</v>
+      </c>
+      <c r="K24" s="0">
+        <v>423.33029621400868</v>
+      </c>
+      <c r="L24" s="0">
+        <v>0.88414253263824893</v>
+      </c>
+      <c r="M24" s="0">
+        <v>0.11585746736175108</v>
+      </c>
+      <c r="N24" s="0">
+        <v>0.91203886564785608</v>
+      </c>
+      <c r="O24" s="0">
+        <v>-75.726879399764101</v>
+      </c>
+      <c r="P24" s="0">
+        <v>114.95713592325546</v>
+      </c>
+      <c r="Q24" s="0">
+        <v>39.23025652349137</v>
+      </c>
+      <c r="R24" s="0">
+        <v>74.901448200781559</v>
+      </c>
+      <c r="S24" s="0">
+        <v>461.71072469425599</v>
+      </c>
+      <c r="T24" s="0">
+        <v>642.1488290984089</v>
+      </c>
+      <c r="U24" s="0">
+        <v>740.26972640437634</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>4</v>
+      </c>
+      <c r="B25" s="0">
+        <v>1</v>
+      </c>
+      <c r="C25" s="0">
+        <v>15</v>
+      </c>
+      <c r="D25" s="0">
+        <v>51.825064679478217</v>
+      </c>
+      <c r="E25" s="0">
+        <v>576.27516495942029</v>
+      </c>
+      <c r="F25" s="0">
+        <v>205.81742929112625</v>
+      </c>
+      <c r="G25" s="0">
+        <v>56.998883955324231</v>
+      </c>
+      <c r="H25" s="0">
+        <v>34.971395564619314</v>
+      </c>
+      <c r="I25" s="0">
+        <v>8.0297204800564597</v>
+      </c>
+      <c r="J25" s="0">
+        <v>423.32078747809578</v>
+      </c>
+      <c r="K25" s="0">
+        <v>423.33029621400868</v>
+      </c>
+      <c r="L25" s="0">
+        <v>0.88414253263824893</v>
+      </c>
+      <c r="M25" s="0">
+        <v>0.11585746736175108</v>
+      </c>
+      <c r="N25" s="0">
+        <v>0.91203886564785608</v>
+      </c>
+      <c r="O25" s="0">
+        <v>-75.726879399764101</v>
+      </c>
+      <c r="P25" s="0">
+        <v>114.95713592325546</v>
+      </c>
+      <c r="Q25" s="0">
+        <v>39.23025652349137</v>
+      </c>
+      <c r="R25" s="0">
+        <v>74.901448200781559</v>
+      </c>
+      <c r="S25" s="0">
+        <v>461.71072469425599</v>
+      </c>
+      <c r="T25" s="0">
+        <v>642.1488290984089</v>
+      </c>
+      <c r="U25" s="0">
+        <v>740.26972640437634</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>4</v>
+      </c>
+      <c r="B26" s="0">
+        <v>2</v>
+      </c>
+      <c r="C26" s="0">
+        <v>200</v>
+      </c>
+      <c r="D26" s="0">
+        <v>40.274014252055466</v>
+      </c>
+      <c r="E26" s="0">
+        <v>187.80654055743616</v>
+      </c>
+      <c r="F26" s="0">
+        <v>160.22280478768698</v>
+      </c>
+      <c r="G26" s="0">
+        <v>51.732066573263879</v>
+      </c>
+      <c r="H26" s="0">
+        <v>39.258781543621069</v>
+      </c>
+      <c r="I26" s="0">
+        <v>9.009151883115047</v>
+      </c>
+      <c r="J26" s="0">
+        <v>334.62137079610983</v>
+      </c>
+      <c r="K26" s="0">
+        <v>335.83004539008448</v>
+      </c>
+      <c r="L26" s="0">
+        <v>0.97227100017591717</v>
+      </c>
+      <c r="M26" s="0">
+        <v>0.027728999824082834</v>
+      </c>
+      <c r="N26" s="0">
+        <v>0.94178044055143995</v>
+      </c>
+      <c r="O26" s="0">
+        <v>-75.72842307261476</v>
+      </c>
+      <c r="P26" s="0">
+        <v>96.633452863376959</v>
+      </c>
+      <c r="Q26" s="0">
+        <v>20.905029790762196</v>
+      </c>
+      <c r="R26" s="0">
+        <v>124.052495517411</v>
+      </c>
+      <c r="S26" s="0">
+        <v>299.50625310685882</v>
+      </c>
+      <c r="T26" s="0">
+        <v>366.06246921662841</v>
+      </c>
+      <c r="U26" s="0">
+        <v>427.14435696349483</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0">
+        <v>4</v>
+      </c>
+      <c r="B27" s="0">
+        <v>2</v>
+      </c>
+      <c r="C27" s="0">
+        <v>300</v>
+      </c>
+      <c r="D27" s="0">
+        <v>38.631671909763959</v>
+      </c>
+      <c r="E27" s="0">
+        <v>159.41640260872009</v>
+      </c>
+      <c r="F27" s="0">
+        <v>163.30723752801896</v>
+      </c>
+      <c r="G27" s="0">
+        <v>48.765203276508714</v>
+      </c>
+      <c r="H27" s="0">
+        <v>41.907742000414295</v>
+      </c>
+      <c r="I27" s="0">
+        <v>9.3270547230769871</v>
+      </c>
+      <c r="J27" s="0">
+        <v>305.90929773248263</v>
+      </c>
+      <c r="K27" s="0">
+        <v>312.31961408600864</v>
+      </c>
+      <c r="L27" s="0">
+        <v>0.99962149322780525</v>
+      </c>
+      <c r="M27" s="0">
+        <v>0.00037850677219475326</v>
+      </c>
+      <c r="N27" s="0">
+        <v>0.95025792016389776</v>
+      </c>
+      <c r="O27" s="0">
+        <v>-75.728465647123997</v>
+      </c>
+      <c r="P27" s="0">
+        <v>95.487487591009938</v>
+      </c>
+      <c r="Q27" s="0">
+        <v>19.759021943885948</v>
+      </c>
+      <c r="R27" s="0">
+        <v>115.55841560203844</v>
+      </c>
+      <c r="S27" s="0">
+        <v>260.77261967734194</v>
+      </c>
+      <c r="T27" s="0">
+        <v>326.6976001095336</v>
+      </c>
+      <c r="U27" s="0">
+        <v>388.98012460368045</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0">
+        <v>0</v>
+      </c>
+      <c r="B28" s="0">
+        <v>2</v>
+      </c>
+      <c r="C28" s="0">
+        <v>200</v>
+      </c>
+      <c r="D28" s="0">
+        <v>37.000638184882597</v>
+      </c>
+      <c r="E28" s="0">
+        <v>179.82731426700303</v>
+      </c>
+      <c r="F28" s="0">
+        <v>153.41997806300787</v>
+      </c>
+      <c r="G28" s="0">
+        <v>45.231204514215605</v>
+      </c>
+      <c r="H28" s="0">
+        <v>45.364591356696423</v>
+      </c>
+      <c r="I28" s="0">
+        <v>9.4042041290879848</v>
+      </c>
+      <c r="J28" s="0">
+        <v>251.38849041531856</v>
+      </c>
+      <c r="K28" s="0">
+        <v>251.44705246971833</v>
+      </c>
+      <c r="L28" s="0">
+        <v>0.90983344087702944</v>
+      </c>
+      <c r="M28" s="0">
+        <v>0.090166559122970558</v>
+      </c>
+      <c r="N28" s="0">
+        <v>0.95789965300735824</v>
+      </c>
+      <c r="O28" s="0">
+        <v>-75.740978230225579</v>
+      </c>
+      <c r="P28" s="0">
+        <v>89.733510525939892</v>
+      </c>
+      <c r="Q28" s="0">
+        <v>13.992532295714312</v>
+      </c>
+      <c r="R28" s="0">
+        <v>103.34164352297101</v>
+      </c>
+      <c r="S28" s="0">
+        <v>233.84412117084503</v>
+      </c>
+      <c r="T28" s="0">
+        <v>262.15829456207211</v>
+      </c>
+      <c r="U28" s="0">
+        <v>288.89203945888221</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0">
+        <v>4</v>
+      </c>
+      <c r="B29" s="0">
+        <v>2</v>
+      </c>
+      <c r="C29" s="0">
+        <v>200</v>
+      </c>
+      <c r="D29" s="0">
+        <v>38.462416408453919</v>
+      </c>
+      <c r="E29" s="0">
+        <v>178.15455181366258</v>
+      </c>
+      <c r="F29" s="0">
+        <v>154.33744399454736</v>
+      </c>
+      <c r="G29" s="0">
+        <v>48.046211841692674</v>
+      </c>
+      <c r="H29" s="0">
+        <v>42.629208672731359</v>
+      </c>
+      <c r="I29" s="0">
+        <v>9.3245794855759634</v>
+      </c>
+      <c r="J29" s="0">
+        <v>343.86945106473837</v>
+      </c>
+      <c r="K29" s="0">
+        <v>344.05646235301128</v>
+      </c>
+      <c r="L29" s="0">
+        <v>0.99139638908966299</v>
+      </c>
+      <c r="M29" s="0">
+        <v>0.0086036109103370118</v>
+      </c>
+      <c r="N29" s="0">
+        <v>0.94533621830287307</v>
+      </c>
+      <c r="O29" s="0">
+        <v>-75.72842307261476</v>
+      </c>
+      <c r="P29" s="0">
+        <v>96.633452863376959</v>
+      </c>
+      <c r="Q29" s="0">
+        <v>20.905029790762196</v>
+      </c>
+      <c r="R29" s="0">
+        <v>124.052495517411</v>
+      </c>
+      <c r="S29" s="0">
+        <v>299.50625310685882</v>
+      </c>
+      <c r="T29" s="0">
+        <v>366.06246921662841</v>
+      </c>
+      <c r="U29" s="0">
+        <v>427.14435696349483</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0">
+        <v>0</v>
+      </c>
+      <c r="B30" s="0">
+        <v>2</v>
+      </c>
+      <c r="C30" s="0">
+        <v>200</v>
+      </c>
+      <c r="D30" s="0">
+        <v>37.000638184882597</v>
+      </c>
+      <c r="E30" s="0">
+        <v>179.82731426700303</v>
+      </c>
+      <c r="F30" s="0">
+        <v>153.41997806300787</v>
+      </c>
+      <c r="G30" s="0">
+        <v>45.231204514215605</v>
+      </c>
+      <c r="H30" s="0">
+        <v>45.364591356696423</v>
+      </c>
+      <c r="I30" s="0">
+        <v>9.4042041290879848</v>
+      </c>
+      <c r="J30" s="0">
+        <v>251.38849041531856</v>
+      </c>
+      <c r="K30" s="0">
+        <v>251.44705246971833</v>
+      </c>
+      <c r="L30" s="0">
+        <v>0.90983344087702944</v>
+      </c>
+      <c r="M30" s="0">
+        <v>0.090166559122970558</v>
+      </c>
+      <c r="N30" s="0">
+        <v>0.95789965300735824</v>
+      </c>
+      <c r="O30" s="0">
+        <v>-75.740978230225579</v>
+      </c>
+      <c r="P30" s="0">
+        <v>89.733510525939892</v>
+      </c>
+      <c r="Q30" s="0">
+        <v>13.992532295714312</v>
+      </c>
+      <c r="R30" s="0">
+        <v>103.34164352297101</v>
+      </c>
+      <c r="S30" s="0">
+        <v>233.84412117084503</v>
+      </c>
+      <c r="T30" s="0">
+        <v>262.15829456207211</v>
+      </c>
+      <c r="U30" s="0">
+        <v>288.89203945888221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>